<commit_message>
updated files in questionnaire_data folder
</commit_message>
<xml_diff>
--- a/questionnaire_data/questionnaire_analysis.xlsx
+++ b/questionnaire_data/questionnaire_analysis.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/arnaldpuy/Documents/papers/topology_risk_models/code_topology_risk_models/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/oxr092@student.bham.ac.uk/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72D4173E-E5DA-EB48-A51A-32386F3C1EC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3449BCFD-7303-2540-973F-CCD9436BA556}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="620" windowWidth="38400" windowHeight="18360" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1_TidyData" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="888" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="889" uniqueCount="196">
   <si>
     <t>Model</t>
   </si>
@@ -130,9 +130,6 @@
     <t>InitializeRealize → initialize2 → hist_addfld1d → allhistfldlist_make_active</t>
   </si>
   <si>
-    <t>There have been several questions where the path involves hist_addfld1d(). That's the only function in any of these paths I have any familiarity with, so I'm probably giving the same answers for all of these.</t>
-  </si>
-  <si>
     <t>lnd _init → initialize2 → hist_addfld1d → allhistfldlist_addfld → get proc bounds</t>
   </si>
   <si>
@@ -175,15 +172,9 @@
     <t>Moderately familiar</t>
   </si>
   <si>
-    <t>main_ftcs is a new code developed by one of my colleagues. It enables more flexible river simulation, including bifurcation. Because I didn't code this, I'm not as familiar as main_human.</t>
-  </si>
-  <si>
     <t>main_human → read_result → read_binary</t>
   </si>
   <si>
-    <t>Read_binary is the fundamental function to read binary files. read_result is, I regret giving it this name, a function to read time series files.  Reading files is truly a fundamental process in simulation.</t>
-  </si>
-  <si>
     <t>main_ftcs → read_result → read_binary</t>
   </si>
   <si>
@@ -223,9 +214,6 @@
     <t>prog_hlf2one → conv_r1tor2</t>
   </si>
   <si>
-    <t>I don't remember prog_hlf2one.f very well, but it must convert data spatial resolutions from half-degree to one-degree.</t>
-  </si>
-  <si>
     <t>prog_map_C05 → conv_r2tor1</t>
   </si>
   <si>
@@ -235,9 +223,6 @@
     <t>prog_frcgw → wrte_ascii2</t>
   </si>
   <si>
-    <t>This program generates files the fraction of groundwater to the total water withdrawal. wrte_ascii2 is a function to generate a national list of quantities. I don't remember well what list is output with this process.</t>
-  </si>
-  <si>
     <t>htuscale → conv_r2tor1</t>
   </si>
   <si>
@@ -323,9 +308,6 @@
   </si>
   <si>
     <t>parameter.get_parameter → dataset2double</t>
-  </si>
-  <si>
-    <t>This was also already discussed. The whole exercise becomes somewhat annoying.</t>
   </si>
   <si>
     <t>update_riverflow → routing_cascade → linear_cascade</t>
@@ -616,13 +598,53 @@
   </si>
   <si>
     <t>Mean (Q1–Q4)</t>
+  </si>
+  <si>
+    <t>There have been several questions where the path involves hist_addfld1d(). […] I'm probably giving the same answers for all of these.</t>
+  </si>
+  <si>
+    <r>
+      <t>main_ftcs is a new code</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> […]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> It enables more flexible river simulation, including bifurcation. […]</t>
+    </r>
+  </si>
+  <si>
+    <t>Read_binary is the fundamental function to read binary files. read_result is […] a function to read time series files. Reading files is truly a fundamental process in simulation.</t>
+  </si>
+  <si>
+    <t>[…] prog_hlf2one.f […] it must convert data spatial resolutions from half-degree to one-degree.</t>
+  </si>
+  <si>
+    <t>This program generates files the fraction of groundwater to the total water withdrawal. wrte_ascii2 is a function to generate a national list of quantities. […]</t>
+  </si>
+  <si>
+    <t>This was also already discussed […]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOTE: Within the free-text comments, any identifable information (e.g. words or sentences that once patched together could narrow down the identity of the respondent, specific contributions to a model's code etc.) have been removed and replaced with […] to ensure anonymity of the respondants </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -635,21 +657,31 @@
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="9"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="9"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
       <color rgb="FF2C3E50"/>
       <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="11">
@@ -1081,7 +1113,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N108"/>
+  <dimension ref="A1:N110"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -2128,7 +2160,7 @@
       </c>
       <c r="N26" s="2"/>
     </row>
-    <row r="27" spans="1:14" ht="39" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:14" ht="26" x14ac:dyDescent="0.2">
       <c r="A27" s="3" t="s">
         <v>14</v>
       </c>
@@ -2169,7 +2201,7 @@
         <v>0</v>
       </c>
       <c r="N27" s="3" t="s">
-        <v>33</v>
+        <v>189</v>
       </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.2">
@@ -2225,7 +2257,7 @@
         <v>10</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E29" s="3" t="s">
         <v>17</v>
@@ -2267,7 +2299,7 @@
         <v>10</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>17</v>
@@ -2309,7 +2341,7 @@
         <v>10</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E31" s="3" t="s">
         <v>17</v>
@@ -2351,10 +2383,10 @@
         <v>11</v>
       </c>
       <c r="D32" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="E32" s="4" t="s">
         <v>35</v>
-      </c>
-      <c r="E32" s="4" t="s">
-        <v>36</v>
       </c>
       <c r="F32" s="4" t="s">
         <v>23</v>
@@ -2383,10 +2415,10 @@
         <v>11</v>
       </c>
       <c r="D33" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="E33" s="4" t="s">
         <v>35</v>
-      </c>
-      <c r="E33" s="4" t="s">
-        <v>36</v>
       </c>
       <c r="F33" s="4" t="s">
         <v>23</v>
@@ -2415,10 +2447,10 @@
         <v>11</v>
       </c>
       <c r="D34" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="E34" s="4" t="s">
         <v>35</v>
-      </c>
-      <c r="E34" s="4" t="s">
-        <v>36</v>
       </c>
       <c r="F34" s="4" t="s">
         <v>23</v>
@@ -2447,10 +2479,10 @@
         <v>12</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F35" s="4" t="s">
         <v>23</v>
@@ -2479,10 +2511,10 @@
         <v>12</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F36" s="4" t="s">
         <v>23</v>
@@ -2511,10 +2543,10 @@
         <v>12</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F37" s="4" t="s">
         <v>23</v>
@@ -2543,10 +2575,10 @@
         <v>13</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F38" s="4" t="s">
         <v>23</v>
@@ -2575,10 +2607,10 @@
         <v>13</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F39" s="4" t="s">
         <v>23</v>
@@ -2607,10 +2639,10 @@
         <v>13</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F40" s="4" t="s">
         <v>23</v>
@@ -2639,13 +2671,13 @@
         <v>14</v>
       </c>
       <c r="D41" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="E41" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="F41" s="5" t="s">
         <v>39</v>
-      </c>
-      <c r="E41" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="F41" s="5" t="s">
-        <v>40</v>
       </c>
       <c r="G41" s="5">
         <v>4</v>
@@ -2681,10 +2713,10 @@
         <v>14</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E42" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F42" s="4" t="s">
         <v>23</v>
@@ -2713,10 +2745,10 @@
         <v>14</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E43" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F43" s="4" t="s">
         <v>23</v>
@@ -2745,10 +2777,10 @@
         <v>15</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F44" s="6" t="s">
         <v>27</v>
@@ -2787,10 +2819,10 @@
         <v>15</v>
       </c>
       <c r="D45" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E45" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F45" s="5" t="s">
         <v>18</v>
@@ -2829,10 +2861,10 @@
         <v>15</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F46" s="6" t="s">
         <v>18</v>
@@ -2862,22 +2894,22 @@
     </row>
     <row r="47" spans="1:14" ht="65" x14ac:dyDescent="0.2">
       <c r="A47" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B47" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B47" s="3" t="s">
+      <c r="C47" s="3">
+        <v>1</v>
+      </c>
+      <c r="D47" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="C47" s="3">
-        <v>1</v>
-      </c>
-      <c r="D47" s="3" t="s">
-        <v>44</v>
-      </c>
       <c r="E47" s="3" t="s">
         <v>17</v>
       </c>
       <c r="F47" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G47" s="3">
         <v>4</v>
@@ -2901,27 +2933,27 @@
         <v>0</v>
       </c>
       <c r="N47" s="3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="48" spans="1:14" ht="26" x14ac:dyDescent="0.2">
+      <c r="A48" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C48" s="2">
+        <v>2</v>
+      </c>
+      <c r="D48" s="2" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="48" spans="1:14" ht="39" x14ac:dyDescent="0.2">
-      <c r="A48" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="B48" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C48" s="2">
-        <v>2</v>
-      </c>
-      <c r="D48" s="2" t="s">
+      <c r="E48" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F48" s="2" t="s">
         <v>46</v>
-      </c>
-      <c r="E48" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F48" s="2" t="s">
-        <v>47</v>
       </c>
       <c r="G48" s="2">
         <v>3</v>
@@ -2945,27 +2977,27 @@
         <v>0</v>
       </c>
       <c r="N48" s="2" t="s">
-        <v>48</v>
+        <v>190</v>
       </c>
     </row>
     <row r="49" spans="1:14" ht="39" x14ac:dyDescent="0.2">
       <c r="A49" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B49" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B49" s="3" t="s">
-        <v>43</v>
-      </c>
       <c r="C49" s="3">
         <v>3</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E49" s="3" t="s">
         <v>17</v>
       </c>
       <c r="F49" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G49" s="3">
         <v>4</v>
@@ -2989,27 +3021,27 @@
         <v>0</v>
       </c>
       <c r="N49" s="3" t="s">
-        <v>50</v>
+        <v>191</v>
       </c>
     </row>
     <row r="50" spans="1:14" ht="26" x14ac:dyDescent="0.2">
       <c r="A50" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B50" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B50" s="2" t="s">
-        <v>43</v>
-      </c>
       <c r="C50" s="2">
         <v>4</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="E50" s="2" t="s">
         <v>17</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G50" s="2">
         <v>3</v>
@@ -3033,27 +3065,27 @@
         <v>0</v>
       </c>
       <c r="N50" s="2" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A51" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B51" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B51" s="3" t="s">
-        <v>43</v>
-      </c>
       <c r="C51" s="3">
         <v>5</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="E51" s="3" t="s">
         <v>17</v>
       </c>
       <c r="F51" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G51" s="3">
         <v>4</v>
@@ -3080,22 +3112,22 @@
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A52" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B52" s="2" t="s">
         <v>42</v>
-      </c>
-      <c r="B52" s="2" t="s">
-        <v>43</v>
       </c>
       <c r="C52" s="2">
         <v>6</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E52" s="2" t="s">
         <v>17</v>
       </c>
       <c r="F52" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G52" s="2">
         <v>3</v>
@@ -3122,22 +3154,22 @@
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A53" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B53" s="3" t="s">
         <v>42</v>
-      </c>
-      <c r="B53" s="3" t="s">
-        <v>43</v>
       </c>
       <c r="C53" s="3">
         <v>7</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="E53" s="3" t="s">
         <v>17</v>
       </c>
       <c r="F53" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G53" s="3">
         <v>4</v>
@@ -3161,27 +3193,27 @@
         <v>0</v>
       </c>
       <c r="N53" s="3" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="54" spans="1:14" ht="26" x14ac:dyDescent="0.2">
       <c r="A54" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B54" s="2" t="s">
         <v>42</v>
-      </c>
-      <c r="B54" s="2" t="s">
-        <v>43</v>
       </c>
       <c r="C54" s="2">
         <v>8</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E54" s="2" t="s">
         <v>17</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G54" s="2">
         <v>4</v>
@@ -3205,27 +3237,27 @@
         <v>0</v>
       </c>
       <c r="N54" s="2" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A55" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B55" s="3" t="s">
         <v>42</v>
-      </c>
-      <c r="B55" s="3" t="s">
-        <v>43</v>
       </c>
       <c r="C55" s="3">
         <v>9</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E55" s="3" t="s">
         <v>17</v>
       </c>
       <c r="F55" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G55" s="3">
         <v>3</v>
@@ -3252,22 +3284,22 @@
     </row>
     <row r="56" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A56" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B56" s="2" t="s">
         <v>42</v>
-      </c>
-      <c r="B56" s="2" t="s">
-        <v>43</v>
       </c>
       <c r="C56" s="2">
         <v>10</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E56" s="2" t="s">
         <v>17</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G56" s="2">
         <v>3</v>
@@ -3294,22 +3326,22 @@
     </row>
     <row r="57" spans="1:14" ht="39" x14ac:dyDescent="0.2">
       <c r="A57" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B57" s="5" t="s">
         <v>42</v>
-      </c>
-      <c r="B57" s="5" t="s">
-        <v>43</v>
       </c>
       <c r="C57" s="5">
         <v>11</v>
       </c>
       <c r="D57" s="5" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="E57" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F57" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G57" s="5">
         <v>4</v>
@@ -3333,24 +3365,24 @@
         <v>0</v>
       </c>
       <c r="N57" s="5" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="58" spans="1:14" ht="26" x14ac:dyDescent="0.2">
       <c r="A58" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B58" s="6" t="s">
         <v>42</v>
-      </c>
-      <c r="B58" s="6" t="s">
-        <v>43</v>
       </c>
       <c r="C58" s="6">
         <v>12</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F58" s="6" t="s">
         <v>18</v>
@@ -3377,27 +3409,27 @@
         <v>0</v>
       </c>
       <c r="N58" s="6" t="s">
-        <v>64</v>
+        <v>192</v>
       </c>
     </row>
     <row r="59" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A59" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B59" s="5" t="s">
         <v>42</v>
-      </c>
-      <c r="B59" s="5" t="s">
-        <v>43</v>
       </c>
       <c r="C59" s="5">
         <v>13</v>
       </c>
       <c r="D59" s="5" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="E59" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F59" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G59" s="5">
         <v>4</v>
@@ -3421,27 +3453,27 @@
         <v>0</v>
       </c>
       <c r="N59" s="5" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
     </row>
     <row r="60" spans="1:14" ht="39" x14ac:dyDescent="0.2">
       <c r="A60" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B60" s="6" t="s">
         <v>42</v>
-      </c>
-      <c r="B60" s="6" t="s">
-        <v>43</v>
       </c>
       <c r="C60" s="6">
         <v>14</v>
       </c>
       <c r="D60" s="6" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="E60" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F60" s="6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G60" s="6">
         <v>3</v>
@@ -3465,27 +3497,27 @@
         <v>0</v>
       </c>
       <c r="N60" s="6" t="s">
-        <v>68</v>
+        <v>193</v>
       </c>
     </row>
     <row r="61" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A61" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B61" s="5" t="s">
         <v>42</v>
-      </c>
-      <c r="B61" s="5" t="s">
-        <v>43</v>
       </c>
       <c r="C61" s="5">
         <v>15</v>
       </c>
       <c r="D61" s="5" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="E61" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F61" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G61" s="5">
         <v>4</v>
@@ -3509,27 +3541,27 @@
         <v>0</v>
       </c>
       <c r="N61" s="5" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
     </row>
     <row r="62" spans="1:14" ht="52" x14ac:dyDescent="0.2">
       <c r="A62" s="2" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C62" s="2">
         <v>1</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="E62" s="2" t="s">
         <v>17</v>
       </c>
       <c r="F62" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G62" s="2">
         <v>4</v>
@@ -3553,27 +3585,27 @@
         <v>0</v>
       </c>
       <c r="N62" s="2" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="63" spans="1:14" ht="26" x14ac:dyDescent="0.2">
       <c r="A63" s="3" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C63" s="3">
         <v>2</v>
       </c>
       <c r="D63" s="3" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="E63" s="3" t="s">
         <v>17</v>
       </c>
       <c r="F63" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G63" s="3">
         <v>4</v>
@@ -3597,27 +3629,27 @@
         <v>0</v>
       </c>
       <c r="N63" s="3" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
     </row>
     <row r="64" spans="1:14" ht="26" x14ac:dyDescent="0.2">
       <c r="A64" s="2" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B64" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C64" s="2">
+        <v>3</v>
+      </c>
+      <c r="D64" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="C64" s="2">
-        <v>3</v>
-      </c>
-      <c r="D64" s="2" t="s">
-        <v>77</v>
-      </c>
       <c r="E64" s="2" t="s">
         <v>17</v>
       </c>
       <c r="F64" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G64" s="2">
         <v>4</v>
@@ -3641,27 +3673,27 @@
         <v>0</v>
       </c>
       <c r="N64" s="2" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
     </row>
     <row r="65" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A65" s="3" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C65" s="3">
         <v>4</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="E65" s="3" t="s">
         <v>17</v>
       </c>
       <c r="F65" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G65" s="3">
         <v>4</v>
@@ -3685,27 +3717,27 @@
         <v>0</v>
       </c>
       <c r="N65" s="3" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
     </row>
     <row r="66" spans="1:14" ht="26" x14ac:dyDescent="0.2">
       <c r="A66" s="2" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C66" s="2">
         <v>5</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="E66" s="2" t="s">
         <v>17</v>
       </c>
       <c r="F66" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G66" s="2">
         <v>4</v>
@@ -3729,27 +3761,27 @@
         <v>0</v>
       </c>
       <c r="N66" s="2" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
     </row>
     <row r="67" spans="1:14" ht="26" x14ac:dyDescent="0.2">
       <c r="A67" s="3" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C67" s="3">
         <v>6</v>
       </c>
       <c r="D67" s="3" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E67" s="3" t="s">
         <v>17</v>
       </c>
       <c r="F67" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G67" s="3">
         <v>4</v>
@@ -3773,27 +3805,27 @@
         <v>0</v>
       </c>
       <c r="N67" s="3" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
     </row>
     <row r="68" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A68" s="2" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C68" s="2">
         <v>7</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="E68" s="2" t="s">
         <v>17</v>
       </c>
       <c r="F68" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G68" s="2">
         <v>4</v>
@@ -3817,27 +3849,27 @@
         <v>0</v>
       </c>
       <c r="N68" s="2" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
     </row>
     <row r="69" spans="1:14" ht="26" x14ac:dyDescent="0.2">
       <c r="A69" s="3" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C69" s="3">
         <v>8</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="E69" s="3" t="s">
         <v>17</v>
       </c>
       <c r="F69" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G69" s="3">
         <v>4</v>
@@ -3861,27 +3893,27 @@
         <v>0</v>
       </c>
       <c r="N69" s="3" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
     </row>
     <row r="70" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A70" s="2" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C70" s="2">
         <v>9</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="E70" s="2" t="s">
         <v>17</v>
       </c>
       <c r="F70" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G70" s="2">
         <v>4</v>
@@ -3905,27 +3937,27 @@
         <v>0</v>
       </c>
       <c r="N70" s="2" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
     </row>
     <row r="71" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A71" s="3" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C71" s="3">
         <v>10</v>
       </c>
       <c r="D71" s="3" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="E71" s="3" t="s">
         <v>17</v>
       </c>
       <c r="F71" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G71" s="3">
         <v>4</v>
@@ -3949,27 +3981,27 @@
         <v>0</v>
       </c>
       <c r="N71" s="3" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
     </row>
     <row r="72" spans="1:14" ht="26" x14ac:dyDescent="0.2">
       <c r="A72" s="6" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B72" s="6" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C72" s="6">
         <v>11</v>
       </c>
       <c r="D72" s="6" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="E72" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F72" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G72" s="6">
         <v>4</v>
@@ -3993,27 +4025,27 @@
         <v>0</v>
       </c>
       <c r="N72" s="6" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
     </row>
     <row r="73" spans="1:14" ht="26" x14ac:dyDescent="0.2">
       <c r="A73" s="5" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B73" s="5" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C73" s="5">
         <v>12</v>
       </c>
       <c r="D73" s="5" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="E73" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F73" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G73" s="5">
         <v>4</v>
@@ -4037,27 +4069,27 @@
         <v>0</v>
       </c>
       <c r="N73" s="5" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="74" spans="1:14" ht="26" x14ac:dyDescent="0.2">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="74" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A74" s="6" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B74" s="6" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C74" s="6">
         <v>13</v>
       </c>
       <c r="D74" s="6" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="E74" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F74" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G74" s="6">
         <v>4</v>
@@ -4081,27 +4113,27 @@
         <v>0</v>
       </c>
       <c r="N74" s="6" t="s">
-        <v>98</v>
+        <v>194</v>
       </c>
     </row>
     <row r="75" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A75" s="5" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B75" s="5" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C75" s="5">
         <v>14</v>
       </c>
       <c r="D75" s="5" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="E75" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F75" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G75" s="5">
         <v>4</v>
@@ -4128,22 +4160,22 @@
     </row>
     <row r="76" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A76" s="6" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B76" s="6" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C76" s="6">
         <v>15</v>
       </c>
       <c r="D76" s="6" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="E76" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F76" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G76" s="6">
         <v>4</v>
@@ -4170,22 +4202,22 @@
     </row>
     <row r="77" spans="1:14" ht="39" x14ac:dyDescent="0.2">
       <c r="A77" s="3" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="C77" s="3">
         <v>1</v>
       </c>
       <c r="D77" s="3" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="E77" s="3" t="s">
         <v>17</v>
       </c>
       <c r="F77" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G77" s="3">
         <v>3</v>
@@ -4209,27 +4241,27 @@
         <v>0</v>
       </c>
       <c r="N77" s="3" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
     </row>
     <row r="78" spans="1:14" ht="52" x14ac:dyDescent="0.2">
       <c r="A78" s="2" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="C78" s="2">
         <v>2</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="E78" s="2" t="s">
         <v>17</v>
       </c>
       <c r="F78" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G78" s="2">
         <v>3</v>
@@ -4253,27 +4285,27 @@
         <v>0</v>
       </c>
       <c r="N78" s="2" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
     </row>
     <row r="79" spans="1:14" ht="39" x14ac:dyDescent="0.2">
       <c r="A79" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="B79" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="C79" s="3">
+        <v>3</v>
+      </c>
+      <c r="D79" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="B79" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="C79" s="3">
-        <v>3</v>
-      </c>
-      <c r="D79" s="3" t="s">
-        <v>107</v>
-      </c>
       <c r="E79" s="3" t="s">
         <v>17</v>
       </c>
       <c r="F79" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G79" s="3">
         <v>3</v>
@@ -4297,27 +4329,27 @@
         <v>0</v>
       </c>
       <c r="N79" s="3" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
     </row>
     <row r="80" spans="1:14" ht="39" x14ac:dyDescent="0.2">
       <c r="A80" s="2" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="C80" s="2">
         <v>4</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="E80" s="2" t="s">
         <v>17</v>
       </c>
       <c r="F80" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G80" s="2">
         <v>3</v>
@@ -4344,22 +4376,22 @@
     </row>
     <row r="81" spans="1:14" ht="52" x14ac:dyDescent="0.2">
       <c r="A81" s="3" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B81" s="3" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="C81" s="3">
         <v>5</v>
       </c>
       <c r="D81" s="3" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="E81" s="3" t="s">
         <v>17</v>
       </c>
       <c r="F81" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G81" s="3">
         <v>3</v>
@@ -4386,22 +4418,22 @@
     </row>
     <row r="82" spans="1:14" ht="52" x14ac:dyDescent="0.2">
       <c r="A82" s="2" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="C82" s="2">
         <v>6</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="E82" s="2" t="s">
         <v>17</v>
       </c>
       <c r="F82" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G82" s="2">
         <v>3</v>
@@ -4425,27 +4457,27 @@
         <v>0</v>
       </c>
       <c r="N82" s="2" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
     </row>
     <row r="83" spans="1:14" ht="39" x14ac:dyDescent="0.2">
       <c r="A83" s="3" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B83" s="3" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="C83" s="3">
         <v>7</v>
       </c>
       <c r="D83" s="3" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="E83" s="3" t="s">
         <v>17</v>
       </c>
       <c r="F83" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G83" s="3">
         <v>3</v>
@@ -4472,22 +4504,22 @@
     </row>
     <row r="84" spans="1:14" ht="39" x14ac:dyDescent="0.2">
       <c r="A84" s="2" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="C84" s="2">
         <v>8</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="E84" s="2" t="s">
         <v>17</v>
       </c>
       <c r="F84" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G84" s="2">
         <v>3</v>
@@ -4514,22 +4546,22 @@
     </row>
     <row r="85" spans="1:14" ht="39" x14ac:dyDescent="0.2">
       <c r="A85" s="3" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B85" s="3" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="C85" s="3">
         <v>9</v>
       </c>
       <c r="D85" s="3" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="E85" s="3" t="s">
         <v>17</v>
       </c>
       <c r="F85" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G85" s="3">
         <v>3</v>
@@ -4556,22 +4588,22 @@
     </row>
     <row r="86" spans="1:14" ht="52" x14ac:dyDescent="0.2">
       <c r="A86" s="2" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="C86" s="2">
         <v>10</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="E86" s="2" t="s">
         <v>17</v>
       </c>
       <c r="F86" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G86" s="2">
         <v>3</v>
@@ -4598,19 +4630,19 @@
     </row>
     <row r="87" spans="1:14" ht="39" x14ac:dyDescent="0.2">
       <c r="A87" s="5" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B87" s="5" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="C87" s="5">
         <v>11</v>
       </c>
       <c r="D87" s="5" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="E87" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F87" s="5" t="s">
         <v>18</v>
@@ -4637,27 +4669,27 @@
         <v>0</v>
       </c>
       <c r="N87" s="5" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
     </row>
     <row r="88" spans="1:14" ht="26" x14ac:dyDescent="0.2">
       <c r="A88" s="6" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B88" s="6" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="C88" s="6">
         <v>12</v>
       </c>
       <c r="D88" s="6" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="E88" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F88" s="6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G88" s="6">
         <v>3</v>
@@ -4684,19 +4716,19 @@
     </row>
     <row r="89" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A89" s="5" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B89" s="5" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="C89" s="5">
         <v>13</v>
       </c>
       <c r="D89" s="5" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="E89" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F89" s="5" t="s">
         <v>18</v>
@@ -4726,22 +4758,22 @@
     </row>
     <row r="90" spans="1:14" ht="26" x14ac:dyDescent="0.2">
       <c r="A90" s="6" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B90" s="6" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="C90" s="6">
         <v>14</v>
       </c>
       <c r="D90" s="6" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="E90" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F90" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G90" s="6">
         <v>4</v>
@@ -4768,22 +4800,22 @@
     </row>
     <row r="91" spans="1:14" ht="26" x14ac:dyDescent="0.2">
       <c r="A91" s="5" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B91" s="5" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="C91" s="5">
         <v>15</v>
       </c>
       <c r="D91" s="5" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="E91" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F91" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G91" s="5">
         <v>3</v>
@@ -4810,22 +4842,22 @@
     </row>
     <row r="92" spans="1:14" ht="26" x14ac:dyDescent="0.2">
       <c r="A92" s="2" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="C92" s="2">
         <v>1</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="E92" s="2" t="s">
         <v>17</v>
       </c>
       <c r="F92" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G92" s="2">
         <v>4</v>
@@ -4849,27 +4881,27 @@
         <v>0</v>
       </c>
       <c r="N92" s="2" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
     </row>
     <row r="93" spans="1:14" ht="26" x14ac:dyDescent="0.2">
       <c r="A93" s="3" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="B93" s="3" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="C93" s="3">
         <v>2</v>
       </c>
       <c r="D93" s="3" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="E93" s="3" t="s">
         <v>17</v>
       </c>
       <c r="F93" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G93" s="3">
         <v>4</v>
@@ -4893,27 +4925,27 @@
         <v>0</v>
       </c>
       <c r="N93" s="3" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
     </row>
     <row r="94" spans="1:14" ht="26" x14ac:dyDescent="0.2">
       <c r="A94" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B94" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C94" s="2">
+        <v>3</v>
+      </c>
+      <c r="D94" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="B94" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="C94" s="2">
-        <v>3</v>
-      </c>
-      <c r="D94" s="2" t="s">
-        <v>129</v>
-      </c>
       <c r="E94" s="2" t="s">
         <v>17</v>
       </c>
       <c r="F94" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G94" s="2">
         <v>3</v>
@@ -4937,27 +4969,27 @@
         <v>0</v>
       </c>
       <c r="N94" s="2" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
     </row>
     <row r="95" spans="1:14" ht="26" x14ac:dyDescent="0.2">
       <c r="A95" s="3" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="B95" s="3" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="C95" s="3">
         <v>4</v>
       </c>
       <c r="D95" s="3" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="E95" s="3" t="s">
         <v>17</v>
       </c>
       <c r="F95" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G95" s="3">
         <v>3</v>
@@ -4981,27 +5013,27 @@
         <v>0</v>
       </c>
       <c r="N95" s="3" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
     </row>
     <row r="96" spans="1:14" ht="26" x14ac:dyDescent="0.2">
       <c r="A96" s="2" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="C96" s="2">
         <v>5</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="E96" s="2" t="s">
         <v>17</v>
       </c>
       <c r="F96" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G96" s="2">
         <v>4</v>
@@ -5025,27 +5057,27 @@
         <v>0</v>
       </c>
       <c r="N96" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
     </row>
     <row r="97" spans="1:14" ht="39" x14ac:dyDescent="0.2">
       <c r="A97" s="3" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="B97" s="3" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="C97" s="3">
         <v>6</v>
       </c>
       <c r="D97" s="3" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="E97" s="3" t="s">
         <v>17</v>
       </c>
       <c r="F97" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G97" s="3">
         <v>4</v>
@@ -5069,27 +5101,27 @@
         <v>0</v>
       </c>
       <c r="N97" s="3" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
     </row>
     <row r="98" spans="1:14" ht="26" x14ac:dyDescent="0.2">
       <c r="A98" s="2" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="C98" s="2">
         <v>7</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="E98" s="2" t="s">
         <v>17</v>
       </c>
       <c r="F98" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G98" s="2">
         <v>4</v>
@@ -5113,27 +5145,27 @@
         <v>0</v>
       </c>
       <c r="N98" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
     </row>
     <row r="99" spans="1:14" ht="52" x14ac:dyDescent="0.2">
       <c r="A99" s="3" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="B99" s="3" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="C99" s="3">
         <v>8</v>
       </c>
       <c r="D99" s="3" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="E99" s="3" t="s">
         <v>17</v>
       </c>
       <c r="F99" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G99" s="3">
         <v>4</v>
@@ -5157,27 +5189,27 @@
         <v>0</v>
       </c>
       <c r="N99" s="3" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
     </row>
     <row r="100" spans="1:14" ht="39" x14ac:dyDescent="0.2">
       <c r="A100" s="2" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="C100" s="2">
         <v>9</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="E100" s="2" t="s">
         <v>17</v>
       </c>
       <c r="F100" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G100" s="2">
         <v>4</v>
@@ -5201,27 +5233,27 @@
         <v>0</v>
       </c>
       <c r="N100" s="2" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
     </row>
     <row r="101" spans="1:14" ht="26" x14ac:dyDescent="0.2">
       <c r="A101" s="3" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="B101" s="3" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="C101" s="3">
         <v>10</v>
       </c>
       <c r="D101" s="3" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="E101" s="3" t="s">
         <v>17</v>
       </c>
       <c r="F101" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G101" s="3">
         <v>4</v>
@@ -5245,27 +5277,27 @@
         <v>0</v>
       </c>
       <c r="N101" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
     </row>
     <row r="102" spans="1:14" ht="26" x14ac:dyDescent="0.2">
       <c r="A102" s="6" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="B102" s="6" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="C102" s="6">
         <v>11</v>
       </c>
       <c r="D102" s="6" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="E102" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F102" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G102" s="6">
         <v>4</v>
@@ -5289,27 +5321,27 @@
         <v>0</v>
       </c>
       <c r="N102" s="6" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
     </row>
     <row r="103" spans="1:14" ht="26" x14ac:dyDescent="0.2">
       <c r="A103" s="5" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="B103" s="5" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="C103" s="5">
         <v>12</v>
       </c>
       <c r="D103" s="5" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="E103" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F103" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G103" s="5">
         <v>4</v>
@@ -5333,27 +5365,27 @@
         <v>0</v>
       </c>
       <c r="N103" s="5" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
     </row>
     <row r="104" spans="1:14" ht="26" x14ac:dyDescent="0.2">
       <c r="A104" s="6" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="B104" s="6" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="C104" s="6">
         <v>13</v>
       </c>
       <c r="D104" s="6" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="E104" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F104" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G104" s="6">
         <v>4</v>
@@ -5377,27 +5409,27 @@
         <v>0</v>
       </c>
       <c r="N104" s="6" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
     </row>
     <row r="105" spans="1:14" ht="26" x14ac:dyDescent="0.2">
       <c r="A105" s="5" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="B105" s="5" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="C105" s="5">
         <v>14</v>
       </c>
       <c r="D105" s="5" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="E105" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F105" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G105" s="5">
         <v>4</v>
@@ -5421,27 +5453,27 @@
         <v>0</v>
       </c>
       <c r="N105" s="5" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
     </row>
     <row r="106" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A106" s="6" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="B106" s="6" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="C106" s="6">
         <v>15</v>
       </c>
       <c r="D106" s="6" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="E106" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F106" s="6" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="G106" s="6"/>
       <c r="H106" s="6"/>
@@ -5456,16 +5488,21 @@
     </row>
     <row r="108" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A108" s="7" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="B108" s="8" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="C108" s="9" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="D108" s="10" t="s">
-        <v>154</v>
+        <v>148</v>
+      </c>
+    </row>
+    <row r="110" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A110" t="s">
+        <v>195</v>
       </c>
     </row>
   </sheetData>
@@ -5491,7 +5528,7 @@
   <sheetData>
     <row r="1" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="18" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -5513,34 +5550,34 @@
         <v>2</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="J2" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E2" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="L2" s="1" t="s">
         <v>158</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.2">
@@ -5663,7 +5700,7 @@
         <v>4</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="D6" s="12" t="s">
         <v>17</v>
@@ -5701,7 +5738,7 @@
         <v>5</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="D7" s="11" t="s">
         <v>17</v>
@@ -5887,7 +5924,7 @@
         <v>10</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="D12" s="12" t="s">
         <v>17</v>
@@ -5925,10 +5962,10 @@
         <v>14</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E13" s="13">
         <v>1</v>
@@ -5961,10 +5998,10 @@
         <v>15</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E14" s="14">
         <v>3</v>
@@ -5993,13 +6030,13 @@
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A15" s="11" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B15" s="11">
         <v>1</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D15" s="11" t="s">
         <v>17</v>
@@ -6029,13 +6066,13 @@
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16" s="12" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B16" s="12">
         <v>2</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D16" s="12" t="s">
         <v>17</v>
@@ -6065,13 +6102,13 @@
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17" s="11" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B17" s="11">
         <v>3</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D17" s="11" t="s">
         <v>17</v>
@@ -6101,13 +6138,13 @@
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A18" s="12" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B18" s="12">
         <v>4</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D18" s="12" t="s">
         <v>17</v>
@@ -6137,13 +6174,13 @@
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19" s="11" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B19" s="11">
         <v>5</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D19" s="11" t="s">
         <v>17</v>
@@ -6173,13 +6210,13 @@
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A20" s="12" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B20" s="12">
         <v>6</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D20" s="12" t="s">
         <v>17</v>
@@ -6209,13 +6246,13 @@
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A21" s="11" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B21" s="11">
         <v>7</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="D21" s="11" t="s">
         <v>17</v>
@@ -6245,13 +6282,13 @@
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A22" s="12" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B22" s="12">
         <v>8</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="D22" s="12" t="s">
         <v>17</v>
@@ -6281,13 +6318,13 @@
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A23" s="11" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B23" s="11">
         <v>9</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="D23" s="11" t="s">
         <v>17</v>
@@ -6317,13 +6354,13 @@
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A24" s="12" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B24" s="12">
         <v>10</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="D24" s="12" t="s">
         <v>17</v>
@@ -6353,16 +6390,16 @@
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A25" s="13" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B25" s="13">
         <v>11</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="D25" s="13" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E25" s="13">
         <v>1</v>
@@ -6389,16 +6426,16 @@
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A26" s="14" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B26" s="14">
         <v>12</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D26" s="14" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E26" s="14">
         <v>1</v>
@@ -6425,16 +6462,16 @@
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A27" s="13" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B27" s="13">
         <v>13</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="D27" s="13" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E27" s="13">
         <v>1</v>
@@ -6461,16 +6498,16 @@
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A28" s="14" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B28" s="14">
         <v>14</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="D28" s="14" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E28" s="14">
         <v>1</v>
@@ -6497,16 +6534,16 @@
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A29" s="13" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B29" s="13">
         <v>15</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="D29" s="13" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E29" s="13">
         <v>1</v>
@@ -6533,13 +6570,13 @@
     </row>
     <row r="30" spans="1:12" ht="26" x14ac:dyDescent="0.2">
       <c r="A30" s="12" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B30" s="12">
         <v>1</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="D30" s="12" t="s">
         <v>17</v>
@@ -6569,13 +6606,13 @@
     </row>
     <row r="31" spans="1:12" ht="26" x14ac:dyDescent="0.2">
       <c r="A31" s="11" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B31" s="11">
         <v>2</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="D31" s="11" t="s">
         <v>17</v>
@@ -6605,13 +6642,13 @@
     </row>
     <row r="32" spans="1:12" ht="26" x14ac:dyDescent="0.2">
       <c r="A32" s="12" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B32" s="12">
         <v>3</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="D32" s="12" t="s">
         <v>17</v>
@@ -6641,13 +6678,13 @@
     </row>
     <row r="33" spans="1:12" ht="26" x14ac:dyDescent="0.2">
       <c r="A33" s="11" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B33" s="11">
         <v>4</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="D33" s="11" t="s">
         <v>17</v>
@@ -6677,13 +6714,13 @@
     </row>
     <row r="34" spans="1:12" ht="26" x14ac:dyDescent="0.2">
       <c r="A34" s="12" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B34" s="12">
         <v>5</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="D34" s="12" t="s">
         <v>17</v>
@@ -6713,13 +6750,13 @@
     </row>
     <row r="35" spans="1:12" ht="26" x14ac:dyDescent="0.2">
       <c r="A35" s="11" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B35" s="11">
         <v>6</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="D35" s="11" t="s">
         <v>17</v>
@@ -6749,13 +6786,13 @@
     </row>
     <row r="36" spans="1:12" ht="26" x14ac:dyDescent="0.2">
       <c r="A36" s="12" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B36" s="12">
         <v>7</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="D36" s="12" t="s">
         <v>17</v>
@@ -6785,13 +6822,13 @@
     </row>
     <row r="37" spans="1:12" ht="26" x14ac:dyDescent="0.2">
       <c r="A37" s="11" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B37" s="11">
         <v>8</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="D37" s="11" t="s">
         <v>17</v>
@@ -6821,13 +6858,13 @@
     </row>
     <row r="38" spans="1:12" ht="26" x14ac:dyDescent="0.2">
       <c r="A38" s="12" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B38" s="12">
         <v>9</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="D38" s="12" t="s">
         <v>17</v>
@@ -6857,13 +6894,13 @@
     </row>
     <row r="39" spans="1:12" ht="26" x14ac:dyDescent="0.2">
       <c r="A39" s="11" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B39" s="11">
         <v>10</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="D39" s="11" t="s">
         <v>17</v>
@@ -6893,16 +6930,16 @@
     </row>
     <row r="40" spans="1:12" ht="26" x14ac:dyDescent="0.2">
       <c r="A40" s="14" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B40" s="14">
         <v>11</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="D40" s="14" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E40" s="14">
         <v>1</v>
@@ -6929,16 +6966,16 @@
     </row>
     <row r="41" spans="1:12" ht="26" x14ac:dyDescent="0.2">
       <c r="A41" s="13" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B41" s="13">
         <v>12</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="D41" s="13" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E41" s="13">
         <v>1</v>
@@ -6965,16 +7002,16 @@
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A42" s="14" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B42" s="14">
         <v>13</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="D42" s="14" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E42" s="14">
         <v>1</v>
@@ -7001,16 +7038,16 @@
     </row>
     <row r="43" spans="1:12" ht="26" x14ac:dyDescent="0.2">
       <c r="A43" s="13" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B43" s="13">
         <v>14</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="D43" s="13" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E43" s="13">
         <v>1</v>
@@ -7037,16 +7074,16 @@
     </row>
     <row r="44" spans="1:12" ht="26" x14ac:dyDescent="0.2">
       <c r="A44" s="14" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B44" s="14">
         <v>15</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="D44" s="14" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E44" s="14">
         <v>1</v>
@@ -7073,13 +7110,13 @@
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A45" s="11" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B45" s="11">
         <v>1</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="D45" s="11" t="s">
         <v>17</v>
@@ -7109,13 +7146,13 @@
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A46" s="12" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B46" s="12">
         <v>2</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="D46" s="12" t="s">
         <v>17</v>
@@ -7145,13 +7182,13 @@
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A47" s="11" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B47" s="11">
         <v>3</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="D47" s="11" t="s">
         <v>17</v>
@@ -7181,13 +7218,13 @@
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A48" s="12" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B48" s="12">
         <v>4</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="D48" s="12" t="s">
         <v>17</v>
@@ -7217,13 +7254,13 @@
     </row>
     <row r="49" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A49" s="11" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B49" s="11">
         <v>5</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="D49" s="11" t="s">
         <v>17</v>
@@ -7253,13 +7290,13 @@
     </row>
     <row r="50" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A50" s="12" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B50" s="12">
         <v>6</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="D50" s="12" t="s">
         <v>17</v>
@@ -7289,13 +7326,13 @@
     </row>
     <row r="51" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A51" s="11" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B51" s="11">
         <v>7</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="D51" s="11" t="s">
         <v>17</v>
@@ -7325,13 +7362,13 @@
     </row>
     <row r="52" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A52" s="12" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B52" s="12">
         <v>8</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="D52" s="12" t="s">
         <v>17</v>
@@ -7361,13 +7398,13 @@
     </row>
     <row r="53" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A53" s="11" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B53" s="11">
         <v>9</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="D53" s="11" t="s">
         <v>17</v>
@@ -7397,13 +7434,13 @@
     </row>
     <row r="54" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A54" s="12" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B54" s="12">
         <v>10</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="D54" s="12" t="s">
         <v>17</v>
@@ -7433,16 +7470,16 @@
     </row>
     <row r="55" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A55" s="13" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B55" s="13">
         <v>11</v>
       </c>
       <c r="C55" s="5" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="D55" s="13" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E55" s="13">
         <v>1</v>
@@ -7469,16 +7506,16 @@
     </row>
     <row r="56" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A56" s="14" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B56" s="14">
         <v>12</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="D56" s="14" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E56" s="14">
         <v>1</v>
@@ -7505,16 +7542,16 @@
     </row>
     <row r="57" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A57" s="13" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B57" s="13">
         <v>13</v>
       </c>
       <c r="C57" s="5" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="D57" s="13" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E57" s="13">
         <v>1</v>
@@ -7541,16 +7578,16 @@
     </row>
     <row r="58" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A58" s="14" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B58" s="14">
         <v>14</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="D58" s="14" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E58" s="14">
         <v>1</v>
@@ -7577,16 +7614,16 @@
     </row>
     <row r="59" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A59" s="13" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B59" s="13">
         <v>15</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="D59" s="13" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E59" s="13">
         <v>1</v>
@@ -7613,13 +7650,13 @@
     </row>
     <row r="60" spans="1:12" ht="26" x14ac:dyDescent="0.2">
       <c r="A60" s="12" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="B60" s="12">
         <v>1</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="D60" s="12" t="s">
         <v>17</v>
@@ -7649,13 +7686,13 @@
     </row>
     <row r="61" spans="1:12" ht="26" x14ac:dyDescent="0.2">
       <c r="A61" s="11" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="B61" s="11">
         <v>2</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="D61" s="11" t="s">
         <v>17</v>
@@ -7685,13 +7722,13 @@
     </row>
     <row r="62" spans="1:12" ht="26" x14ac:dyDescent="0.2">
       <c r="A62" s="12" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="B62" s="12">
         <v>3</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="D62" s="12" t="s">
         <v>17</v>
@@ -7721,13 +7758,13 @@
     </row>
     <row r="63" spans="1:12" ht="26" x14ac:dyDescent="0.2">
       <c r="A63" s="11" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="B63" s="11">
         <v>4</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="D63" s="11" t="s">
         <v>17</v>
@@ -7757,13 +7794,13 @@
     </row>
     <row r="64" spans="1:12" ht="26" x14ac:dyDescent="0.2">
       <c r="A64" s="12" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="B64" s="12">
         <v>5</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="D64" s="12" t="s">
         <v>17</v>
@@ -7793,13 +7830,13 @@
     </row>
     <row r="65" spans="1:12" ht="26" x14ac:dyDescent="0.2">
       <c r="A65" s="11" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="B65" s="11">
         <v>6</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="D65" s="11" t="s">
         <v>17</v>
@@ -7829,13 +7866,13 @@
     </row>
     <row r="66" spans="1:12" ht="26" x14ac:dyDescent="0.2">
       <c r="A66" s="12" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="B66" s="12">
         <v>7</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="D66" s="12" t="s">
         <v>17</v>
@@ -7865,13 +7902,13 @@
     </row>
     <row r="67" spans="1:12" ht="26" x14ac:dyDescent="0.2">
       <c r="A67" s="11" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="B67" s="11">
         <v>8</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="D67" s="11" t="s">
         <v>17</v>
@@ -7901,13 +7938,13 @@
     </row>
     <row r="68" spans="1:12" ht="26" x14ac:dyDescent="0.2">
       <c r="A68" s="12" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="B68" s="12">
         <v>9</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="D68" s="12" t="s">
         <v>17</v>
@@ -7937,13 +7974,13 @@
     </row>
     <row r="69" spans="1:12" ht="26" x14ac:dyDescent="0.2">
       <c r="A69" s="11" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="B69" s="11">
         <v>10</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="D69" s="11" t="s">
         <v>17</v>
@@ -7973,16 +8010,16 @@
     </row>
     <row r="70" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A70" s="14" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="B70" s="14">
         <v>11</v>
       </c>
       <c r="C70" s="6" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="D70" s="14" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E70" s="14">
         <v>1</v>
@@ -8009,16 +8046,16 @@
     </row>
     <row r="71" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A71" s="13" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="B71" s="13">
         <v>12</v>
       </c>
       <c r="C71" s="5" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="D71" s="13" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E71" s="13">
         <v>1</v>
@@ -8045,16 +8082,16 @@
     </row>
     <row r="72" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A72" s="14" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="B72" s="14">
         <v>13</v>
       </c>
       <c r="C72" s="6" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="D72" s="14" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E72" s="14">
         <v>1</v>
@@ -8081,16 +8118,16 @@
     </row>
     <row r="73" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A73" s="13" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="B73" s="13">
         <v>14</v>
       </c>
       <c r="C73" s="5" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="D73" s="13" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E73" s="13">
         <v>1</v>
@@ -8117,16 +8154,16 @@
     </row>
     <row r="74" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A74" s="14" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="B74" s="14">
         <v>15</v>
       </c>
       <c r="C74" s="6" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="D74" s="14" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E74" s="14">
         <v>0</v>
@@ -8178,7 +8215,7 @@
   <sheetData>
     <row r="1" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="18" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -8194,39 +8231,39 @@
     </row>
     <row r="2" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>182</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>183</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>184</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>187</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" s="15" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="C3" s="15">
         <v>63</v>
@@ -8252,10 +8289,10 @@
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" s="15" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="C4" s="15">
         <v>63</v>
@@ -8281,10 +8318,10 @@
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" s="15" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="C5" s="15">
         <v>63</v>
@@ -8310,10 +8347,10 @@
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" s="15" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="C6" s="15">
         <v>63</v>
@@ -8339,10 +8376,10 @@
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" s="15" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C7" s="15">
         <v>63</v>
@@ -8371,7 +8408,7 @@
         <v>14</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="C8" s="16">
         <v>23</v>
@@ -8400,7 +8437,7 @@
         <v>14</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="C9" s="16">
         <v>23</v>
@@ -8429,7 +8466,7 @@
         <v>14</v>
       </c>
       <c r="B10" s="17" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="C10" s="17">
         <v>23</v>
@@ -8458,7 +8495,7 @@
         <v>14</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="C11" s="16">
         <v>23</v>
@@ -8487,7 +8524,7 @@
         <v>14</v>
       </c>
       <c r="B12" s="17" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C12" s="17">
         <v>23</v>
@@ -8513,10 +8550,10 @@
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A13" s="17" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B13" s="17" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="C13" s="17">
         <v>10</v>
@@ -8542,10 +8579,10 @@
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14" s="17" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B14" s="17" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="C14" s="17">
         <v>10</v>
@@ -8571,10 +8608,10 @@
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A15" s="16" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="C15" s="16">
         <v>10</v>
@@ -8600,10 +8637,10 @@
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16" s="17" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B16" s="17" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="C16" s="17">
         <v>10</v>
@@ -8629,10 +8666,10 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A17" s="16" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B17" s="16" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C17" s="16">
         <v>10</v>
@@ -8658,10 +8695,10 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A18" s="16" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B18" s="16" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="C18" s="16">
         <v>10</v>
@@ -8687,10 +8724,10 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A19" s="16" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B19" s="16" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="C19" s="16">
         <v>10</v>
@@ -8716,10 +8753,10 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A20" s="17" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B20" s="17" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="C20" s="17">
         <v>10</v>
@@ -8745,10 +8782,10 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A21" s="16" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B21" s="16" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="C21" s="16">
         <v>10</v>
@@ -8774,10 +8811,10 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A22" s="17" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B22" s="17" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C22" s="17">
         <v>10</v>
@@ -8803,10 +8840,10 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A23" s="17" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B23" s="17" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="C23" s="17">
         <v>10</v>
@@ -8832,10 +8869,10 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A24" s="17" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B24" s="17" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="C24" s="17">
         <v>10</v>
@@ -8861,10 +8898,10 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A25" s="16" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B25" s="16" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="C25" s="16">
         <v>10</v>
@@ -8890,10 +8927,10 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A26" s="17" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B26" s="17" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="C26" s="17">
         <v>10</v>
@@ -8919,10 +8956,10 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A27" s="16" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B27" s="16" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C27" s="16">
         <v>10</v>
@@ -8948,10 +8985,10 @@
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A28" s="16" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="B28" s="16" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="C28" s="16">
         <v>10</v>
@@ -8977,10 +9014,10 @@
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A29" s="16" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="B29" s="16" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="C29" s="16">
         <v>10</v>
@@ -9006,10 +9043,10 @@
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A30" s="17" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="B30" s="17" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="C30" s="17">
         <v>10</v>
@@ -9035,10 +9072,10 @@
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A31" s="16" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="B31" s="16" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="C31" s="16">
         <v>10</v>
@@ -9064,10 +9101,10 @@
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A32" s="17" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="B32" s="17" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C32" s="17">
         <v>10</v>

</xml_diff>